<commit_message>
fix(orientation): priorisation CPTS, verbatims cibles MISAS/SSIAD, deduplication et correction explicabilite age
</commit_message>
<xml_diff>
--- a/config/rules/tableau_oria.xlsx
+++ b/config/rules/tableau_oria.xlsx
@@ -1048,7 +1048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB59"/>
+  <dimension ref="A1:AB60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.69921875" defaultRowHeight="13.8"/>
   <cols>
     <col width="22" customWidth="1" style="1" min="1" max="1"/>
@@ -1730,7 +1730,11 @@
       </c>
       <c r="T12" s="5" t="n"/>
       <c r="U12" s="5" t="n"/>
-      <c r="V12" s="11" t="n"/>
+      <c r="V12" s="11" t="inlineStr">
+        <is>
+          <t>La MISAS peut aussi vous accompagner dans la recherche d'un médecin traitant</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1778,7 +1782,11 @@
       </c>
       <c r="T13" s="11" t="n"/>
       <c r="U13" s="11" t="n"/>
-      <c r="V13" s="11" t="n"/>
+      <c r="V13" s="11" t="inlineStr">
+        <is>
+          <t>La MISAS peut aussi vous accompagner dans la recherche d'un médecin traitant</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="27.6" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -4177,6 +4185,33 @@
       <c r="V59" s="11" t="inlineStr">
         <is>
           <t>Envisager une mesure de protection juridique (tutelle, curatelle, sauvegarde de justice) auprès du tribunal de proximité. Retrouvez plus d'informations sur la fiche [Mesures de protection – DAC Var Ouest](https://dac-varouest.fr/index.php/ressources/minformer/mesures-de-protection/).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Santé / Soins</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Accompagnement MISAS pour la recherche de médecin traitant</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>recherche_medecin</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>La MISAS peut aussi vous accompagner dans la recherche d'un médecin traitant</t>
         </is>
       </c>
     </row>

</xml_diff>